<commit_message>
Price check — 03/21/2026
</commit_message>
<xml_diff>
--- a/GITHUBOPENCLAWPRICECHECK.xlsx
+++ b/GITHUBOPENCLAWPRICECHECK.xlsx
@@ -115,15 +115,11 @@
       <alignment vertical="bottom"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment/>
-    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="164" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="165" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="166" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment/>
-    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="167" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="165" fontId="3" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -416,37 +412,38 @@
     <outlinePr summaryBelow="0" summaryRight="0"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L254"/>
+  <dimension ref="A1:M254"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="12.63" defaultRowHeight="15" customHeight="1"/>
   <cols>
     <col width="12.63" customWidth="1" style="11" min="1" max="6"/>
     <col width="14" customWidth="1" style="11" min="7" max="7"/>
     <col width="13" customWidth="1" style="11" min="9" max="10"/>
     <col width="12" customWidth="1" style="11" min="12" max="12"/>
+    <col width="12" customWidth="1" style="11" min="13" max="13"/>
   </cols>
   <sheetData>
     <row r="1" ht="15.75" customHeight="1" s="11">
-      <c r="A1" s="1" t="inlineStr">
+      <c r="A1" s="2" t="inlineStr">
         <is>
           <t>New Price Average</t>
         </is>
       </c>
-      <c r="B1" s="1" t="inlineStr">
+      <c r="B1" s="2" t="inlineStr">
         <is>
           <t>Average vs Listed</t>
         </is>
       </c>
-      <c r="C1" s="1" t="inlineStr">
+      <c r="C1" s="2" t="inlineStr">
         <is>
           <t>#</t>
         </is>
       </c>
-      <c r="D1" s="1" t="inlineStr">
+      <c r="D1" s="2" t="inlineStr">
         <is>
           <t>Item Type</t>
         </is>
       </c>
-      <c r="E1" s="1" t="inlineStr">
+      <c r="E1" s="2" t="inlineStr">
         <is>
           <t>Standard Replacement</t>
         </is>
@@ -456,17 +453,17 @@
           <t>Link</t>
         </is>
       </c>
-      <c r="G1" s="1" t="inlineStr">
+      <c r="G1" s="2" t="inlineStr">
         <is>
           <t>Best Buy SKU</t>
         </is>
       </c>
-      <c r="H1" s="1" t="inlineStr">
+      <c r="H1" s="2" t="inlineStr">
         <is>
           <t>Status / 3/19</t>
         </is>
       </c>
-      <c r="I1" s="1" t="inlineStr">
+      <c r="I1" s="2" t="inlineStr">
         <is>
           <t>Listed Price</t>
         </is>
@@ -482,6 +479,11 @@
       <c r="L1" s="12" t="inlineStr">
         <is>
           <t>3/20</t>
+        </is>
+      </c>
+      <c r="M1" s="12" t="inlineStr">
+        <is>
+          <t>3/21</t>
         </is>
       </c>
     </row>
@@ -492,15 +494,15 @@
       <c r="B2" s="5" t="n">
         <v>0</v>
       </c>
-      <c r="C2" s="1" t="n">
+      <c r="C2" s="2" t="n">
         <v>12</v>
       </c>
-      <c r="D2" s="1" t="inlineStr">
+      <c r="D2" s="2" t="inlineStr">
         <is>
           <t>Audio Player</t>
         </is>
       </c>
-      <c r="E2" s="1" t="inlineStr">
+      <c r="E2" s="2" t="inlineStr">
         <is>
           <t>Insignia - CD Boombox</t>
         </is>
@@ -510,12 +512,12 @@
           <t>https://www.bestbuy.com/site/insignia-insignia-cd-boombox-black/9183279.p?skuId=9183279</t>
         </is>
       </c>
-      <c r="G2" s="1" t="inlineStr">
+      <c r="G2" s="2" t="inlineStr">
         <is>
           <t>9183279</t>
         </is>
       </c>
-      <c r="H2" s="1" t="inlineStr">
+      <c r="H2" s="2" t="inlineStr">
         <is>
           <t>Currently Active</t>
         </is>
@@ -523,7 +525,7 @@
       <c r="I2" s="7" t="n">
         <v>54.99</v>
       </c>
-      <c r="J2" s="1" t="n">
+      <c r="J2" s="2" t="n">
         <v>54.99</v>
       </c>
       <c r="K2" s="4" t="n">
@@ -532,17 +534,20 @@
       <c r="L2" s="13" t="n">
         <v>54.99</v>
       </c>
+      <c r="M2" s="13" t="n">
+        <v>54.99</v>
+      </c>
     </row>
     <row r="3" ht="15.75" customHeight="1" s="11">
-      <c r="C3" s="1" t="n">
+      <c r="C3" s="2" t="n">
         <v>14</v>
       </c>
-      <c r="D3" s="1" t="inlineStr">
+      <c r="D3" s="2" t="inlineStr">
         <is>
           <t>Baby Monitor</t>
         </is>
       </c>
-      <c r="E3" s="1" t="inlineStr">
+      <c r="E3" s="2" t="inlineStr">
         <is>
           <t>VTech Baby Monitor</t>
         </is>
@@ -555,7 +560,7 @@
       <c r="G3" s="8" t="n">
         <v>6624988</v>
       </c>
-      <c r="H3" s="1" t="inlineStr">
+      <c r="H3" s="2" t="inlineStr">
         <is>
           <t>Currently Active</t>
         </is>
@@ -567,6 +572,9 @@
       <c r="L3" s="13" t="n">
         <v>89.95</v>
       </c>
+      <c r="M3" s="13" t="n">
+        <v>89.95</v>
+      </c>
     </row>
     <row r="4" ht="15.75" customHeight="1" s="11">
       <c r="A4" s="4" t="n">
@@ -575,15 +583,15 @@
       <c r="B4" s="5" t="n">
         <v>0</v>
       </c>
-      <c r="C4" s="1" t="n">
+      <c r="C4" s="2" t="n">
         <v>35</v>
       </c>
-      <c r="D4" s="1" t="inlineStr">
+      <c r="D4" s="2" t="inlineStr">
         <is>
           <t>CD Player</t>
         </is>
       </c>
-      <c r="E4" s="1" t="inlineStr">
+      <c r="E4" s="2" t="inlineStr">
         <is>
           <t>Insignia CD Boombox with Built-In Radio</t>
         </is>
@@ -593,12 +601,12 @@
           <t>https://www.bestbuy.com/site/insignia-insignia-cd-boombox-black/9183279.p?skuId=9183279</t>
         </is>
       </c>
-      <c r="G4" s="1" t="inlineStr">
+      <c r="G4" s="2" t="inlineStr">
         <is>
           <t>9183279</t>
         </is>
       </c>
-      <c r="H4" s="1" t="inlineStr">
+      <c r="H4" s="2" t="inlineStr">
         <is>
           <t>Currently Active</t>
         </is>
@@ -606,7 +614,7 @@
       <c r="I4" s="7" t="n">
         <v>54.99</v>
       </c>
-      <c r="J4" s="1" t="n">
+      <c r="J4" s="2" t="n">
         <v>54.99</v>
       </c>
       <c r="K4" s="4" t="n">
@@ -615,17 +623,20 @@
       <c r="L4" s="13" t="n">
         <v>54.99</v>
       </c>
+      <c r="M4" s="13" t="n">
+        <v>54.99</v>
+      </c>
     </row>
     <row r="5" ht="15.75" customHeight="1" s="11">
-      <c r="C5" s="1" t="n">
+      <c r="C5" s="2" t="n">
         <v>67</v>
       </c>
-      <c r="D5" s="1" t="inlineStr">
+      <c r="D5" s="2" t="inlineStr">
         <is>
           <t>Computer</t>
         </is>
       </c>
-      <c r="E5" s="1" t="inlineStr">
+      <c r="E5" s="2" t="inlineStr">
         <is>
           <t>Lenovo IdeaPad Touch-Screen Laptop</t>
         </is>
@@ -638,7 +649,7 @@
       <c r="G5" s="8" t="n">
         <v>11771076</v>
       </c>
-      <c r="H5" s="1" t="inlineStr">
+      <c r="H5" s="2" t="inlineStr">
         <is>
           <t>Currently Active</t>
         </is>
@@ -648,6 +659,11 @@
       </c>
       <c r="J5" s="8" t="n"/>
       <c r="L5" s="14" t="inlineStr">
+        <is>
+          <t>OOS</t>
+        </is>
+      </c>
+      <c r="M5" s="14" t="inlineStr">
         <is>
           <t>OOS</t>
         </is>
@@ -660,15 +676,15 @@
       <c r="B6" s="10" t="n">
         <v>0</v>
       </c>
-      <c r="C6" s="1" t="n">
+      <c r="C6" s="2" t="n">
         <v>98</v>
       </c>
-      <c r="D6" s="1" t="inlineStr">
+      <c r="D6" s="2" t="inlineStr">
         <is>
           <t>Cooktop</t>
         </is>
       </c>
-      <c r="E6" s="1" t="inlineStr">
+      <c r="E6" s="2" t="inlineStr">
         <is>
           <t>Monogram 36" Smart Gas Cooktop</t>
         </is>
@@ -678,12 +694,12 @@
           <t>https://www.bestbuy.com/product/monogram-36-built-in-gas-cooktop-with-5-burners-and-sapphire-glass-precision-knobs-stainless-steel/J7645SJH7H/sku/6089924?utm_source=feed?extStoreId=&amp;ref=212&amp;loc=MajorAppliances&amp;gclsrc=aw.ds&amp;gad_source=1&amp;gad_campaignid=2008</t>
         </is>
       </c>
-      <c r="G6" s="1" t="inlineStr">
+      <c r="G6" s="2" t="inlineStr">
         <is>
           <t>6089924</t>
         </is>
       </c>
-      <c r="H6" s="1" t="inlineStr">
+      <c r="H6" s="2" t="inlineStr">
         <is>
           <t>Currently Active</t>
         </is>
@@ -698,6 +714,9 @@
       <c r="L6" s="13" t="n">
         <v>2900</v>
       </c>
+      <c r="M6" s="13" t="n">
+        <v>2900</v>
+      </c>
     </row>
     <row r="7" ht="15.75" customHeight="1" s="11">
       <c r="A7" s="9" t="n">
@@ -706,15 +725,15 @@
       <c r="B7" s="10" t="n">
         <v>0</v>
       </c>
-      <c r="C7" s="1" t="n">
+      <c r="C7" s="2" t="n">
         <v>121</v>
       </c>
-      <c r="D7" s="1" t="inlineStr">
+      <c r="D7" s="2" t="inlineStr">
         <is>
           <t>Doorbell</t>
         </is>
       </c>
-      <c r="E7" s="1" t="inlineStr">
+      <c r="E7" s="2" t="inlineStr">
         <is>
           <t>Arlo Video Doorbell</t>
         </is>
@@ -724,12 +743,12 @@
           <t>https://www.bestbuy.com/product/arlo-smart-wi-fi-video-doorbell-2nd-generation-wired-battery-operated-with-2k-resolution-white/JJ8QV84GFR/sku/6554331</t>
         </is>
       </c>
-      <c r="G7" s="1" t="inlineStr">
+      <c r="G7" s="2" t="inlineStr">
         <is>
           <t>6554331</t>
         </is>
       </c>
-      <c r="H7" s="1" t="inlineStr">
+      <c r="H7" s="2" t="inlineStr">
         <is>
           <t>Currently Active</t>
         </is>
@@ -744,17 +763,20 @@
       <c r="L7" s="13" t="n">
         <v>49.99</v>
       </c>
+      <c r="M7" s="13" t="n">
+        <v>49.99</v>
+      </c>
     </row>
     <row r="8" ht="15.75" customHeight="1" s="11">
-      <c r="C8" s="1" t="n">
+      <c r="C8" s="2" t="n">
         <v>124</v>
       </c>
-      <c r="D8" s="1" t="inlineStr">
+      <c r="D8" s="2" t="inlineStr">
         <is>
           <t>DVD Player</t>
         </is>
       </c>
-      <c r="E8" s="1" t="inlineStr">
+      <c r="E8" s="2" t="inlineStr">
         <is>
           <t>Panasonic 4K Ultra HD Wi-Fi Blu-Ray Player</t>
         </is>
@@ -767,7 +789,7 @@
       <c r="G8" s="8" t="n">
         <v>6536323</v>
       </c>
-      <c r="H8" s="1" t="inlineStr">
+      <c r="H8" s="2" t="inlineStr">
         <is>
           <t>Currently Active</t>
         </is>
@@ -779,6 +801,9 @@
       <c r="L8" s="13" t="n">
         <v>239.99</v>
       </c>
+      <c r="M8" s="13" t="n">
+        <v>239.99</v>
+      </c>
     </row>
     <row r="9" ht="15.75" customHeight="1" s="11">
       <c r="A9" s="9" t="n">
@@ -787,15 +812,15 @@
       <c r="B9" s="10" t="n">
         <v>0</v>
       </c>
-      <c r="C9" s="1" t="n">
+      <c r="C9" s="2" t="n">
         <v>125</v>
       </c>
-      <c r="D9" s="1" t="inlineStr">
+      <c r="D9" s="2" t="inlineStr">
         <is>
           <t>DVD Player</t>
         </is>
       </c>
-      <c r="E9" s="1" t="inlineStr">
+      <c r="E9" s="2" t="inlineStr">
         <is>
           <t>Sony DVD Player</t>
         </is>
@@ -805,12 +830,12 @@
           <t>https://www.bestbuy.com/site/sony-dvd-player-with-hd-upconversion-black/4790739.p?skuId=4790739</t>
         </is>
       </c>
-      <c r="G9" s="1" t="inlineStr">
+      <c r="G9" s="2" t="inlineStr">
         <is>
           <t>4790739</t>
         </is>
       </c>
-      <c r="H9" s="1" t="inlineStr">
+      <c r="H9" s="2" t="inlineStr">
         <is>
           <t>Currently Active</t>
         </is>
@@ -825,6 +850,9 @@
       <c r="L9" s="13" t="n">
         <v>64.98999999999999</v>
       </c>
+      <c r="M9" s="13" t="n">
+        <v>64.98999999999999</v>
+      </c>
     </row>
     <row r="10" ht="15.75" customHeight="1" s="11">
       <c r="A10" s="9" t="n">
@@ -833,15 +861,15 @@
       <c r="B10" s="10" t="n">
         <v>0</v>
       </c>
-      <c r="C10" s="1" t="n">
+      <c r="C10" s="2" t="n">
         <v>167</v>
       </c>
-      <c r="D10" s="1" t="inlineStr">
+      <c r="D10" s="2" t="inlineStr">
         <is>
           <t>Electric Clock</t>
         </is>
       </c>
-      <c r="E10" s="1" t="inlineStr">
+      <c r="E10" s="2" t="inlineStr">
         <is>
           <t>Sony AM/FM Alarm Clock Radio</t>
         </is>
@@ -851,12 +879,12 @@
           <t>https://www.bestbuy.com/site/sony-am-fm-alarm-clock-radio/6010016.p?skuId=6010016</t>
         </is>
       </c>
-      <c r="G10" s="1" t="inlineStr">
+      <c r="G10" s="2" t="inlineStr">
         <is>
           <t>6010016</t>
         </is>
       </c>
-      <c r="H10" s="1" t="inlineStr">
+      <c r="H10" s="2" t="inlineStr">
         <is>
           <t>Currently Active</t>
         </is>
@@ -871,17 +899,20 @@
       <c r="L10" s="13" t="n">
         <v>39.99</v>
       </c>
+      <c r="M10" s="13" t="n">
+        <v>39.99</v>
+      </c>
     </row>
     <row r="11" ht="15.75" customHeight="1" s="11">
-      <c r="C11" s="1" t="n">
+      <c r="C11" s="2" t="n">
         <v>185</v>
       </c>
-      <c r="D11" s="1" t="inlineStr">
+      <c r="D11" s="2" t="inlineStr">
         <is>
           <t>Electric Wall Oven</t>
         </is>
       </c>
-      <c r="E11" s="1" t="inlineStr">
+      <c r="E11" s="2" t="inlineStr">
         <is>
           <t>GE 24" Electric Single Self-Cleaning Wall Oven</t>
         </is>
@@ -894,7 +925,7 @@
       <c r="G11" s="8" t="n">
         <v>6315212</v>
       </c>
-      <c r="H11" s="1" t="inlineStr">
+      <c r="H11" s="2" t="inlineStr">
         <is>
           <t>Currently Active</t>
         </is>
@@ -906,17 +937,20 @@
       <c r="L11" s="13" t="n">
         <v>1889.99</v>
       </c>
+      <c r="M11" s="13" t="n">
+        <v>1889.99</v>
+      </c>
     </row>
     <row r="12" ht="15.75" customHeight="1" s="11">
-      <c r="C12" s="1" t="n">
+      <c r="C12" s="2" t="n">
         <v>186</v>
       </c>
-      <c r="D12" s="1" t="inlineStr">
+      <c r="D12" s="2" t="inlineStr">
         <is>
           <t>Electric Wall Oven</t>
         </is>
       </c>
-      <c r="E12" s="1" t="inlineStr">
+      <c r="E12" s="2" t="inlineStr">
         <is>
           <t>KitchenAid 24" Electric Convection Wall Oven</t>
         </is>
@@ -929,7 +963,7 @@
       <c r="G12" s="8" t="n">
         <v>6530108</v>
       </c>
-      <c r="H12" s="1" t="inlineStr">
+      <c r="H12" s="2" t="inlineStr">
         <is>
           <t>Currently Active</t>
         </is>
@@ -941,6 +975,9 @@
       <c r="L12" s="13" t="n">
         <v>2654.99</v>
       </c>
+      <c r="M12" s="13" t="n">
+        <v>2654.99</v>
+      </c>
     </row>
     <row r="13" ht="15.75" customHeight="1" s="11">
       <c r="A13" s="4" t="n">
@@ -949,15 +986,15 @@
       <c r="B13" s="5" t="n">
         <v>0</v>
       </c>
-      <c r="C13" s="1" t="n">
+      <c r="C13" s="2" t="n">
         <v>188</v>
       </c>
-      <c r="D13" s="1" t="inlineStr">
+      <c r="D13" s="2" t="inlineStr">
         <is>
           <t>Electric Wall Oven</t>
         </is>
       </c>
-      <c r="E13" s="1" t="inlineStr">
+      <c r="E13" s="2" t="inlineStr">
         <is>
           <t>Bosch 24" Single Electric Convection Wall Oven</t>
         </is>
@@ -967,12 +1004,12 @@
           <t>https://www.bestbuy.com/site/bosch-500-series-24-built-in-single-electric-convection-wall-oven-stainless-steel/6405680.p?skuId=6405680</t>
         </is>
       </c>
-      <c r="G13" s="1" t="inlineStr">
+      <c r="G13" s="2" t="inlineStr">
         <is>
           <t>6405680</t>
         </is>
       </c>
-      <c r="H13" s="1" t="inlineStr">
+      <c r="H13" s="2" t="inlineStr">
         <is>
           <t>Currently Active</t>
         </is>
@@ -980,13 +1017,16 @@
       <c r="I13" s="7" t="n">
         <v>2299.99</v>
       </c>
-      <c r="J13" s="1" t="n">
+      <c r="J13" s="2" t="n">
         <v>2299.99</v>
       </c>
       <c r="K13" s="4" t="n">
         <v>2299.99</v>
       </c>
       <c r="L13" s="13" t="n">
+        <v>2299.99</v>
+      </c>
+      <c r="M13" s="13" t="n">
         <v>2299.99</v>
       </c>
     </row>
@@ -997,15 +1037,15 @@
       <c r="B14" s="5" t="n">
         <v>0</v>
       </c>
-      <c r="C14" s="1" t="n">
+      <c r="C14" s="2" t="n">
         <v>194</v>
       </c>
-      <c r="D14" s="1" t="inlineStr">
+      <c r="D14" s="2" t="inlineStr">
         <is>
           <t>Electric Wall Oven</t>
         </is>
       </c>
-      <c r="E14" s="1" t="inlineStr">
+      <c r="E14" s="2" t="inlineStr">
         <is>
           <t>Bosch 30" Single Electric Wall Oven</t>
         </is>
@@ -1015,12 +1055,12 @@
           <t>https://www.bestbuy.com/site/bosch-500-series-30-built-in-single-electric-convection-wall-oven-stainless-steel/5906157.p?skuId=5906157</t>
         </is>
       </c>
-      <c r="G14" s="1" t="inlineStr">
+      <c r="G14" s="2" t="inlineStr">
         <is>
           <t>5906157</t>
         </is>
       </c>
-      <c r="H14" s="1" t="inlineStr">
+      <c r="H14" s="2" t="inlineStr">
         <is>
           <t>Currently Active</t>
         </is>
@@ -1028,7 +1068,7 @@
       <c r="I14" s="7" t="n">
         <v>2799.99</v>
       </c>
-      <c r="J14" s="1" t="n">
+      <c r="J14" s="2" t="n">
         <v>2799.99</v>
       </c>
       <c r="K14" s="4" t="n">
@@ -1037,17 +1077,20 @@
       <c r="L14" s="13" t="n">
         <v>2799.99</v>
       </c>
+      <c r="M14" s="13" t="n">
+        <v>2799.99</v>
+      </c>
     </row>
     <row r="15" ht="15.75" customHeight="1" s="11">
-      <c r="C15" s="1" t="n">
+      <c r="C15" s="2" t="n">
         <v>209</v>
       </c>
-      <c r="D15" s="1" t="inlineStr">
+      <c r="D15" s="2" t="inlineStr">
         <is>
           <t>Ethernet Switch</t>
         </is>
       </c>
-      <c r="E15" s="1" t="inlineStr">
+      <c r="E15" s="2" t="inlineStr">
         <is>
           <t>Netgear 5 Port Ethernet Switch</t>
         </is>
@@ -1060,7 +1103,7 @@
       <c r="G15" s="8" t="n">
         <v>6040713</v>
       </c>
-      <c r="H15" s="1" t="inlineStr">
+      <c r="H15" s="2" t="inlineStr">
         <is>
           <t>Currently Active</t>
         </is>
@@ -1072,17 +1115,20 @@
       <c r="L15" s="13" t="n">
         <v>39.99</v>
       </c>
+      <c r="M15" s="13" t="n">
+        <v>39.99</v>
+      </c>
     </row>
     <row r="16" ht="15.75" customHeight="1" s="11">
-      <c r="C16" s="1" t="n">
+      <c r="C16" s="2" t="n">
         <v>210</v>
       </c>
-      <c r="D16" s="1" t="inlineStr">
+      <c r="D16" s="2" t="inlineStr">
         <is>
           <t>Ethernet Switch</t>
         </is>
       </c>
-      <c r="E16" s="1" t="inlineStr">
+      <c r="E16" s="2" t="inlineStr">
         <is>
           <t>Netgear 8 Port Ethernet Switch</t>
         </is>
@@ -1095,7 +1141,7 @@
       <c r="G16" s="8" t="n">
         <v>6598710</v>
       </c>
-      <c r="H16" s="1" t="inlineStr">
+      <c r="H16" s="2" t="inlineStr">
         <is>
           <t>Currently Active</t>
         </is>
@@ -1107,17 +1153,20 @@
       <c r="L16" s="13" t="n">
         <v>49.99</v>
       </c>
+      <c r="M16" s="13" t="n">
+        <v>49.99</v>
+      </c>
     </row>
     <row r="17" ht="15.75" customHeight="1" s="11">
-      <c r="C17" s="1" t="n">
+      <c r="C17" s="2" t="n">
         <v>211</v>
       </c>
-      <c r="D17" s="1" t="inlineStr">
+      <c r="D17" s="2" t="inlineStr">
         <is>
           <t>Ethernet Switch</t>
         </is>
       </c>
-      <c r="E17" s="1" t="inlineStr">
+      <c r="E17" s="2" t="inlineStr">
         <is>
           <t>Netgear 24 Port Ethernet Switch</t>
         </is>
@@ -1130,7 +1179,7 @@
       <c r="G17" s="8" t="n">
         <v>6623627</v>
       </c>
-      <c r="H17" s="1" t="inlineStr">
+      <c r="H17" s="2" t="inlineStr">
         <is>
           <t>Currently Active</t>
         </is>
@@ -1142,6 +1191,9 @@
       <c r="L17" s="13" t="n">
         <v>149.99</v>
       </c>
+      <c r="M17" s="13" t="n">
+        <v>149.99</v>
+      </c>
     </row>
     <row r="18" ht="15.75" customHeight="1" s="11">
       <c r="A18" s="9" t="n">
@@ -1150,15 +1202,15 @@
       <c r="B18" s="10" t="n">
         <v>0</v>
       </c>
-      <c r="C18" s="1" t="n">
+      <c r="C18" s="2" t="n">
         <v>212</v>
       </c>
-      <c r="D18" s="1" t="inlineStr">
+      <c r="D18" s="2" t="inlineStr">
         <is>
           <t>Ethernet Switch</t>
         </is>
       </c>
-      <c r="E18" s="1" t="inlineStr">
+      <c r="E18" s="2" t="inlineStr">
         <is>
           <t>Netgear 16 Port Ethernet Switch</t>
         </is>
@@ -1168,12 +1220,12 @@
           <t>https://www.bestbuy.com/product/netgear-16-port-gigabit-unmanaged-ethernet-switch-gray/J2VY7YQ965/sku/6623626?utm_source=feed?extStoreId=1767&amp;ref=212&amp;loc=19621921639&amp;gclsrc=aw.ds&amp;gad_source=4&amp;gad_campaignid=19614357066&amp;gbraid=0AAAAAD-ORIgQ2sB2KmV4w9trYwkg</t>
         </is>
       </c>
-      <c r="G18" s="1" t="inlineStr">
+      <c r="G18" s="2" t="inlineStr">
         <is>
           <t>6623626</t>
         </is>
       </c>
-      <c r="H18" s="1" t="inlineStr">
+      <c r="H18" s="2" t="inlineStr">
         <is>
           <t>Currently Active</t>
         </is>
@@ -1188,6 +1240,9 @@
       <c r="L18" s="13" t="n">
         <v>99.98999999999999</v>
       </c>
+      <c r="M18" s="13" t="n">
+        <v>99.98999999999999</v>
+      </c>
     </row>
     <row r="19" ht="15.75" customHeight="1" s="11">
       <c r="A19" s="9" t="n">
@@ -1196,15 +1251,15 @@
       <c r="B19" s="10" t="n">
         <v>0</v>
       </c>
-      <c r="C19" s="1" t="n">
+      <c r="C19" s="2" t="n">
         <v>224</v>
       </c>
-      <c r="D19" s="1" t="inlineStr">
+      <c r="D19" s="2" t="inlineStr">
         <is>
           <t>Freezer</t>
         </is>
       </c>
-      <c r="E19" s="1" t="inlineStr">
+      <c r="E19" s="2" t="inlineStr">
         <is>
           <t>Insignia 13.8 cu. ft. Upright Freezer</t>
         </is>
@@ -1214,12 +1269,12 @@
           <t>https://www.bestbuy.com/site/insignia-13-8-cu-ft-garage-ready-convertible-upright-freezer-with-energy-star-certification-stainless-steel/6336450.p?skuId=6336450</t>
         </is>
       </c>
-      <c r="G19" s="1" t="inlineStr">
+      <c r="G19" s="2" t="inlineStr">
         <is>
           <t>6336450</t>
         </is>
       </c>
-      <c r="H19" s="1" t="inlineStr">
+      <c r="H19" s="2" t="inlineStr">
         <is>
           <t>Currently Active</t>
         </is>
@@ -1234,23 +1289,26 @@
       <c r="L19" s="13" t="n">
         <v>499.99</v>
       </c>
+      <c r="M19" s="13" t="n">
+        <v>499.99</v>
+      </c>
     </row>
     <row r="20" ht="15.75" customHeight="1" s="11">
-      <c r="A20" s="1" t="n">
+      <c r="A20" s="2" t="n">
         <v>599.99</v>
       </c>
-      <c r="B20" s="1" t="n">
+      <c r="B20" s="2" t="n">
         <v>0</v>
       </c>
-      <c r="C20" s="1" t="n">
+      <c r="C20" s="2" t="n">
         <v>227</v>
       </c>
-      <c r="D20" s="1" t="inlineStr">
+      <c r="D20" s="2" t="inlineStr">
         <is>
           <t>Freezer</t>
         </is>
       </c>
-      <c r="E20" s="1" t="inlineStr">
+      <c r="E20" s="2" t="inlineStr">
         <is>
           <t>Insignia 16 cu. ft. Upright Freezer</t>
         </is>
@@ -1260,12 +1318,12 @@
           <t>https://www.bestbuy.com/site/insignia-17-cu-ft-garage-ready-convertible-upright-freezer-with-energy-star-certification-stainless-steel/6336445.p?skuId=6336445</t>
         </is>
       </c>
-      <c r="G20" s="1" t="inlineStr">
+      <c r="G20" s="2" t="inlineStr">
         <is>
           <t>6336445</t>
         </is>
       </c>
-      <c r="H20" s="1" t="inlineStr">
+      <c r="H20" s="2" t="inlineStr">
         <is>
           <t>Currently Active</t>
         </is>
@@ -1273,11 +1331,14 @@
       <c r="I20" s="7" t="n">
         <v>599.99</v>
       </c>
-      <c r="J20" s="1" t="n">
+      <c r="J20" s="2" t="n">
         <v>599.99</v>
       </c>
-      <c r="K20" s="1" t="n"/>
+      <c r="K20" s="2" t="n"/>
       <c r="L20" s="13" t="n">
+        <v>599.99</v>
+      </c>
+      <c r="M20" s="13" t="n">
         <v>599.99</v>
       </c>
     </row>
@@ -1288,15 +1349,15 @@
       <c r="B21" s="5" t="n">
         <v>0</v>
       </c>
-      <c r="C21" s="1" t="n">
+      <c r="C21" s="2" t="n">
         <v>229</v>
       </c>
-      <c r="D21" s="1" t="inlineStr">
+      <c r="D21" s="2" t="inlineStr">
         <is>
           <t>Freezer</t>
         </is>
       </c>
-      <c r="E21" s="1" t="inlineStr">
+      <c r="E21" s="2" t="inlineStr">
         <is>
           <t>GE 21.3 cu. ft. Upright Freezer</t>
         </is>
@@ -1306,12 +1367,12 @@
           <t>https://www.bestbuy.com/site/ge-21-3-cu-ft-frost-free-upright-freezer-white/5916602.p?skuId=5916602</t>
         </is>
       </c>
-      <c r="G21" s="1" t="inlineStr">
+      <c r="G21" s="2" t="inlineStr">
         <is>
           <t>5916602</t>
         </is>
       </c>
-      <c r="H21" s="1" t="inlineStr">
+      <c r="H21" s="2" t="inlineStr">
         <is>
           <t>Currently Active</t>
         </is>
@@ -1319,13 +1380,16 @@
       <c r="I21" s="7" t="n">
         <v>1049.99</v>
       </c>
-      <c r="J21" s="1" t="n">
+      <c r="J21" s="2" t="n">
         <v>1049.99</v>
       </c>
       <c r="K21" s="4" t="n">
         <v>1049.99</v>
       </c>
       <c r="L21" s="13" t="n">
+        <v>1049.99</v>
+      </c>
+      <c r="M21" s="13" t="n">
         <v>1049.99</v>
       </c>
     </row>
@@ -1336,15 +1400,15 @@
       <c r="B22" s="10" t="n">
         <v>0</v>
       </c>
-      <c r="C22" s="1" t="n">
+      <c r="C22" s="2" t="n">
         <v>231</v>
       </c>
-      <c r="D22" s="1" t="inlineStr">
+      <c r="D22" s="2" t="inlineStr">
         <is>
           <t>Freezer</t>
         </is>
       </c>
-      <c r="E22" s="1" t="inlineStr">
+      <c r="E22" s="2" t="inlineStr">
         <is>
           <t>Amana 16 cu. ft. Chest Freezer</t>
         </is>
@@ -1354,12 +1418,12 @@
           <t>https://www.bestbuy.com/site/amana-16-cu-ft-chest-freezer-with-basket-white/6476505.p?skuId=6476505</t>
         </is>
       </c>
-      <c r="G22" s="1" t="inlineStr">
+      <c r="G22" s="2" t="inlineStr">
         <is>
           <t>6476505</t>
         </is>
       </c>
-      <c r="H22" s="1" t="inlineStr">
+      <c r="H22" s="2" t="inlineStr">
         <is>
           <t>Currently Active</t>
         </is>
@@ -1374,17 +1438,20 @@
       <c r="L22" s="13" t="n">
         <v>639.99</v>
       </c>
+      <c r="M22" s="13" t="n">
+        <v>639.99</v>
+      </c>
     </row>
     <row r="23" ht="15.75" customHeight="1" s="11">
-      <c r="C23" s="1" t="n">
+      <c r="C23" s="2" t="n">
         <v>237</v>
       </c>
-      <c r="D23" s="1" t="inlineStr">
+      <c r="D23" s="2" t="inlineStr">
         <is>
           <t>Gaming Console</t>
         </is>
       </c>
-      <c r="E23" s="1" t="inlineStr">
+      <c r="E23" s="2" t="inlineStr">
         <is>
           <t>Microsoft Xbox Series X Gaming Console</t>
         </is>
@@ -1397,7 +1464,7 @@
       <c r="G23" s="8" t="n">
         <v>6595697</v>
       </c>
-      <c r="H23" s="1" t="inlineStr">
+      <c r="H23" s="2" t="inlineStr">
         <is>
           <t>Currently Active</t>
         </is>
@@ -1409,6 +1476,9 @@
       <c r="L23" s="13" t="n">
         <v>599.99</v>
       </c>
+      <c r="M23" s="13" t="n">
+        <v>599.99</v>
+      </c>
     </row>
     <row r="24" ht="15.75" customHeight="1" s="11">
       <c r="A24" s="9" t="n">
@@ -1417,15 +1487,15 @@
       <c r="B24" s="10" t="n">
         <v>0</v>
       </c>
-      <c r="C24" s="1" t="n">
+      <c r="C24" s="2" t="n">
         <v>241</v>
       </c>
-      <c r="D24" s="1" t="inlineStr">
+      <c r="D24" s="2" t="inlineStr">
         <is>
           <t>Gaming Console</t>
         </is>
       </c>
-      <c r="E24" s="1" t="inlineStr">
+      <c r="E24" s="2" t="inlineStr">
         <is>
           <t>Meta Quest 3 VR Headset</t>
         </is>
@@ -1435,12 +1505,12 @@
           <t>https://www.bestbuy.com/product/meta-quest-3-512gb--virtual-reality-headset-without-wires-thirty-percent-sharper-resolution-2x-graphical-processing-white/J3LHRV8694/sku/6554912?utm_source=feed?extStoreId=894&amp;ref=212&amp;loc=17066407628&amp;gclsrc=aw.ds&amp;gad_source</t>
         </is>
       </c>
-      <c r="G24" s="1" t="inlineStr">
+      <c r="G24" s="2" t="inlineStr">
         <is>
           <t>6554912</t>
         </is>
       </c>
-      <c r="H24" s="1" t="inlineStr">
+      <c r="H24" s="2" t="inlineStr">
         <is>
           <t>Currently Active</t>
         </is>
@@ -1455,17 +1525,20 @@
       <c r="L24" s="13" t="n">
         <v>499.99</v>
       </c>
+      <c r="M24" s="13" t="n">
+        <v>499.99</v>
+      </c>
     </row>
     <row r="25" ht="15.75" customHeight="1" s="11">
-      <c r="C25" s="1" t="n">
+      <c r="C25" s="2" t="n">
         <v>266</v>
       </c>
-      <c r="D25" s="1" t="inlineStr">
+      <c r="D25" s="2" t="inlineStr">
         <is>
           <t>Gas Range</t>
         </is>
       </c>
-      <c r="E25" s="1" t="inlineStr">
+      <c r="E25" s="2" t="inlineStr">
         <is>
           <t>KitchenAid - 5.0 Cu. Ft. Slide-In Gas True Convection Range</t>
         </is>
@@ -1478,7 +1551,7 @@
       <c r="G25" s="8" t="n">
         <v>6640593</v>
       </c>
-      <c r="H25" s="1" t="inlineStr">
+      <c r="H25" s="2" t="inlineStr">
         <is>
           <t>Currently Active</t>
         </is>
@@ -1490,6 +1563,9 @@
       <c r="L25" s="13" t="n">
         <v>2099.99</v>
       </c>
+      <c r="M25" s="13" t="n">
+        <v>2099.99</v>
+      </c>
     </row>
     <row r="26" ht="15.75" customHeight="1" s="11">
       <c r="A26" s="4" t="n">
@@ -1498,15 +1574,15 @@
       <c r="B26" s="5" t="n">
         <v>0</v>
       </c>
-      <c r="C26" s="1" t="n">
+      <c r="C26" s="2" t="n">
         <v>279</v>
       </c>
-      <c r="D26" s="1" t="inlineStr">
+      <c r="D26" s="2" t="inlineStr">
         <is>
           <t>Hard Drive</t>
         </is>
       </c>
-      <c r="E26" s="1" t="inlineStr">
+      <c r="E26" s="2" t="inlineStr">
         <is>
           <t>Western Digital 5TB External Hard Drive</t>
         </is>
@@ -1516,12 +1592,12 @@
           <t>https://www.bestbuy.com/site/wd-easystore-2tb-external-usb-3-2-gen-1-portable-hard-drive-black/6406513.p?skuId=6406513</t>
         </is>
       </c>
-      <c r="G26" s="1" t="inlineStr">
+      <c r="G26" s="2" t="inlineStr">
         <is>
           <t>6406513</t>
         </is>
       </c>
-      <c r="H26" s="1" t="inlineStr">
+      <c r="H26" s="2" t="inlineStr">
         <is>
           <t>Currently Active</t>
         </is>
@@ -1529,13 +1605,16 @@
       <c r="I26" s="7" t="n">
         <v>79.98999999999999</v>
       </c>
-      <c r="J26" s="1" t="n">
+      <c r="J26" s="2" t="n">
         <v>79.98999999999999</v>
       </c>
       <c r="K26" s="4" t="n">
         <v>79.98999999999999</v>
       </c>
       <c r="L26" s="13" t="n">
+        <v>79.98999999999999</v>
+      </c>
+      <c r="M26" s="13" t="n">
         <v>79.98999999999999</v>
       </c>
     </row>
@@ -1546,15 +1625,15 @@
       <c r="B27" s="10" t="n">
         <v>0</v>
       </c>
-      <c r="C27" s="1" t="n">
+      <c r="C27" s="2" t="n">
         <v>308</v>
       </c>
-      <c r="D27" s="1" t="inlineStr">
+      <c r="D27" s="2" t="inlineStr">
         <is>
           <t>Home Phone</t>
         </is>
       </c>
-      <c r="E27" s="1" t="inlineStr">
+      <c r="E27" s="2" t="inlineStr">
         <is>
           <t>AT&amp;T Single Handset Cordless Phone System</t>
         </is>
@@ -1564,12 +1643,12 @@
           <t>https://www.bestbuy.com/site/at-t-crl32102-dect-6-0-expandable-cordless-phone-with-digital-answering-system-and-caller-id-call-waiting-silver/4837076.p?skuId=4837076</t>
         </is>
       </c>
-      <c r="G27" s="1" t="inlineStr">
+      <c r="G27" s="2" t="inlineStr">
         <is>
           <t>4837076</t>
         </is>
       </c>
-      <c r="H27" s="1" t="inlineStr">
+      <c r="H27" s="2" t="inlineStr">
         <is>
           <t>Currently Active</t>
         </is>
@@ -1584,6 +1663,9 @@
       <c r="L27" s="13" t="n">
         <v>64.95</v>
       </c>
+      <c r="M27" s="13" t="n">
+        <v>64.95</v>
+      </c>
     </row>
     <row r="28" ht="15.75" customHeight="1" s="11">
       <c r="A28" s="9" t="n">
@@ -1592,15 +1674,15 @@
       <c r="B28" s="10" t="n">
         <v>0</v>
       </c>
-      <c r="C28" s="1" t="n">
+      <c r="C28" s="2" t="n">
         <v>385</v>
       </c>
-      <c r="D28" s="1" t="inlineStr">
+      <c r="D28" s="2" t="inlineStr">
         <is>
           <t>Modem</t>
         </is>
       </c>
-      <c r="E28" s="1" t="inlineStr">
+      <c r="E28" s="2" t="inlineStr">
         <is>
           <t>ARRIS - SURFboard 32 x 8 Channel Modem</t>
         </is>
@@ -1610,12 +1692,12 @@
           <t>https://www.bestbuy.com/site/arris-surfboard-sb6190-32-x-8-docsis-3-0-cable-modem-white/4600801.p?extStoreId=175&amp;gclid=CjwKCAjwrNmWBhA4EiwAHbjEQDSTZbsuZCaFptZSlJVRm6gA9jXsWH5n6NTA8meFqQA6BuCQe2aHLRoCkcQQAvD_BwE&amp;gclsrc=aw.ds&amp;loc=1&amp;ref=212&amp;skuId=4600801</t>
         </is>
       </c>
-      <c r="G28" s="1" t="inlineStr">
+      <c r="G28" s="2" t="inlineStr">
         <is>
           <t>4600801</t>
         </is>
       </c>
-      <c r="H28" s="1" t="inlineStr">
+      <c r="H28" s="2" t="inlineStr">
         <is>
           <t>Currently Active</t>
         </is>
@@ -1630,17 +1712,20 @@
       <c r="L28" s="13" t="n">
         <v>79</v>
       </c>
+      <c r="M28" s="13" t="n">
+        <v>79</v>
+      </c>
     </row>
     <row r="29" ht="15.75" customHeight="1" s="11">
-      <c r="C29" s="1" t="n">
+      <c r="C29" s="2" t="n">
         <v>386</v>
       </c>
-      <c r="D29" s="1" t="inlineStr">
+      <c r="D29" s="2" t="inlineStr">
         <is>
           <t>Modem</t>
         </is>
       </c>
-      <c r="E29" s="1" t="inlineStr">
+      <c r="E29" s="2" t="inlineStr">
         <is>
           <t>Arris Cable Modem</t>
         </is>
@@ -1653,7 +1738,7 @@
       <c r="G29" s="8" t="n">
         <v>5839003</v>
       </c>
-      <c r="H29" s="1" t="inlineStr">
+      <c r="H29" s="2" t="inlineStr">
         <is>
           <t>Currently Active</t>
         </is>
@@ -1665,6 +1750,9 @@
       <c r="L29" s="13" t="n">
         <v>169</v>
       </c>
+      <c r="M29" s="13" t="n">
+        <v>169</v>
+      </c>
     </row>
     <row r="30" ht="15.75" customHeight="1" s="11">
       <c r="A30" s="9" t="n">
@@ -1673,15 +1761,15 @@
       <c r="B30" s="10" t="n">
         <v>0</v>
       </c>
-      <c r="C30" s="1" t="n">
+      <c r="C30" s="2" t="n">
         <v>387</v>
       </c>
-      <c r="D30" s="1" t="inlineStr">
+      <c r="D30" s="2" t="inlineStr">
         <is>
           <t>Modem-Router Combo</t>
         </is>
       </c>
-      <c r="E30" s="1" t="inlineStr">
+      <c r="E30" s="2" t="inlineStr">
         <is>
           <t>ARRIS - SURFboard Dual-Band Router and 3.0 Cable Modem</t>
         </is>
@@ -1691,12 +1779,12 @@
           <t>https://www.bestbuy.com/product/arris-surfboard-sb6190-32-x-8-docsis-3-0-cable-modem-white/JX7YCY49XC/sku/4600801?utm_source=feed?extStoreId=&amp;ref=212&amp;loc=19618641984&amp;gclsrc=aw.ds&amp;gad_source=1&amp;gad_campaignid=19626707675&amp;gbraid=0AAAAAD-ORIiYcQ7DbnvrhNUEhMxV</t>
         </is>
       </c>
-      <c r="G30" s="1" t="inlineStr">
+      <c r="G30" s="2" t="inlineStr">
         <is>
           <t>4600801</t>
         </is>
       </c>
-      <c r="H30" s="1" t="inlineStr">
+      <c r="H30" s="2" t="inlineStr">
         <is>
           <t>Currently Active</t>
         </is>
@@ -1711,6 +1799,9 @@
       <c r="L30" s="13" t="n">
         <v>79</v>
       </c>
+      <c r="M30" s="13" t="n">
+        <v>79</v>
+      </c>
     </row>
     <row r="31" ht="15.75" customHeight="1" s="11">
       <c r="A31" s="4" t="n">
@@ -1719,15 +1810,15 @@
       <c r="B31" s="5" t="n">
         <v>0</v>
       </c>
-      <c r="C31" s="1" t="n">
+      <c r="C31" s="2" t="n">
         <v>388</v>
       </c>
-      <c r="D31" s="1" t="inlineStr">
+      <c r="D31" s="2" t="inlineStr">
         <is>
           <t>Monitor</t>
         </is>
       </c>
-      <c r="E31" s="1" t="inlineStr">
+      <c r="E31" s="2" t="inlineStr">
         <is>
           <t>Acer 24" Monitor</t>
         </is>
@@ -1737,12 +1828,12 @@
           <t>https://www.bestbuy.com/site/acer-27-ips-led-fhd-120hz-1ms-freesync-monitor-hdmivga-black/6587445.p?skuId=6587445</t>
         </is>
       </c>
-      <c r="G31" s="1" t="inlineStr">
+      <c r="G31" s="2" t="inlineStr">
         <is>
           <t>6587445</t>
         </is>
       </c>
-      <c r="H31" s="1" t="inlineStr">
+      <c r="H31" s="2" t="inlineStr">
         <is>
           <t>Currently Active</t>
         </is>
@@ -1750,13 +1841,16 @@
       <c r="I31" s="7" t="n">
         <v>99.98999999999999</v>
       </c>
-      <c r="J31" s="1" t="n">
+      <c r="J31" s="2" t="n">
         <v>99.98999999999999</v>
       </c>
       <c r="K31" s="4" t="n">
         <v>99.98999999999999</v>
       </c>
       <c r="L31" s="13" t="n">
+        <v>99.98999999999999</v>
+      </c>
+      <c r="M31" s="13" t="n">
         <v>99.98999999999999</v>
       </c>
     </row>
@@ -1767,15 +1861,15 @@
       <c r="B32" s="5" t="n">
         <v>0</v>
       </c>
-      <c r="C32" s="1" t="n">
+      <c r="C32" s="2" t="n">
         <v>443</v>
       </c>
-      <c r="D32" s="1" t="inlineStr">
+      <c r="D32" s="2" t="inlineStr">
         <is>
           <t>Printer</t>
         </is>
       </c>
-      <c r="E32" s="1" t="inlineStr">
+      <c r="E32" s="2" t="inlineStr">
         <is>
           <t>Epson EcoTank Wireless All-in-One Printer</t>
         </is>
@@ -1785,12 +1879,12 @@
           <t>https://www.bestbuy.com/site/epson-ecotank-et-2800-wireless-all-in-one-supertank-inkjet-printer-white/6469371.p?skuId=6469371&amp;extStoreId=894&amp;ref=212&amp;loc=20145591549&amp;gad_source=4</t>
         </is>
       </c>
-      <c r="G32" s="1" t="inlineStr">
+      <c r="G32" s="2" t="inlineStr">
         <is>
           <t>6469371</t>
         </is>
       </c>
-      <c r="H32" s="1" t="inlineStr">
+      <c r="H32" s="2" t="inlineStr">
         <is>
           <t>Currently Active</t>
         </is>
@@ -1798,13 +1892,16 @@
       <c r="I32" s="7" t="n">
         <v>179.99</v>
       </c>
-      <c r="J32" s="1" t="n">
+      <c r="J32" s="2" t="n">
         <v>179.99</v>
       </c>
       <c r="K32" s="4" t="n">
         <v>179.99</v>
       </c>
       <c r="L32" s="13" t="n">
+        <v>179.99</v>
+      </c>
+      <c r="M32" s="13" t="n">
         <v>179.99</v>
       </c>
     </row>
@@ -1815,15 +1912,15 @@
       <c r="B33" s="5" t="n">
         <v>0</v>
       </c>
-      <c r="C33" s="1" t="n">
+      <c r="C33" s="2" t="n">
         <v>445</v>
       </c>
-      <c r="D33" s="1" t="inlineStr">
+      <c r="D33" s="2" t="inlineStr">
         <is>
           <t>Programmable Remote</t>
         </is>
       </c>
-      <c r="E33" s="1" t="inlineStr">
+      <c r="E33" s="2" t="inlineStr">
         <is>
           <t>One for All Universal Remote</t>
         </is>
@@ -1833,12 +1930,12 @@
           <t>https://www.bestbuy.com/site/one-for-all-smart-streamer-universal-remote/6497955.p?skuId=6497955</t>
         </is>
       </c>
-      <c r="G33" s="1" t="inlineStr">
+      <c r="G33" s="2" t="inlineStr">
         <is>
           <t>6497955</t>
         </is>
       </c>
-      <c r="H33" s="1" t="inlineStr">
+      <c r="H33" s="2" t="inlineStr">
         <is>
           <t>Currently Active</t>
         </is>
@@ -1846,13 +1943,16 @@
       <c r="I33" s="7" t="n">
         <v>34.99</v>
       </c>
-      <c r="J33" s="1" t="n">
+      <c r="J33" s="2" t="n">
         <v>34.99</v>
       </c>
       <c r="K33" s="4" t="n">
         <v>34.99</v>
       </c>
       <c r="L33" s="13" t="n">
+        <v>34.99</v>
+      </c>
+      <c r="M33" s="13" t="n">
         <v>34.99</v>
       </c>
     </row>
@@ -1863,15 +1963,15 @@
       <c r="B34" s="5" t="n">
         <v>0</v>
       </c>
-      <c r="C34" s="1" t="n">
+      <c r="C34" s="2" t="n">
         <v>446</v>
       </c>
-      <c r="D34" s="1" t="inlineStr">
+      <c r="D34" s="2" t="inlineStr">
         <is>
           <t>Programmable Remote</t>
         </is>
       </c>
-      <c r="E34" s="1" t="inlineStr">
+      <c r="E34" s="2" t="inlineStr">
         <is>
           <t>Insignia 3-Device Universal Remote</t>
         </is>
@@ -1881,12 +1981,12 @@
           <t>https://www.bestbuy.com/site/insignia-3-device-universal-remote-black/6495829.p?skuId=6495829</t>
         </is>
       </c>
-      <c r="G34" s="1" t="inlineStr">
+      <c r="G34" s="2" t="inlineStr">
         <is>
           <t>6495829</t>
         </is>
       </c>
-      <c r="H34" s="1" t="inlineStr">
+      <c r="H34" s="2" t="inlineStr">
         <is>
           <t>Currently Active</t>
         </is>
@@ -1894,7 +1994,7 @@
       <c r="I34" s="7" t="n">
         <v>19.99</v>
       </c>
-      <c r="J34" s="1" t="n">
+      <c r="J34" s="2" t="n">
         <v>19.99</v>
       </c>
       <c r="K34" s="4" t="n">
@@ -1903,23 +2003,26 @@
       <c r="L34" s="13" t="n">
         <v>19.99</v>
       </c>
+      <c r="M34" s="13" t="n">
+        <v>19.99</v>
+      </c>
     </row>
     <row r="35" ht="15.75" customHeight="1" s="11">
-      <c r="A35" s="1" t="n">
+      <c r="A35" s="2" t="n">
         <v>139.99</v>
       </c>
-      <c r="B35" s="1" t="n">
+      <c r="B35" s="2" t="n">
         <v>0</v>
       </c>
-      <c r="C35" s="1" t="n">
+      <c r="C35" s="2" t="n">
         <v>466</v>
       </c>
-      <c r="D35" s="1" t="inlineStr">
+      <c r="D35" s="2" t="inlineStr">
         <is>
           <t>Router</t>
         </is>
       </c>
-      <c r="E35" s="1" t="inlineStr">
+      <c r="E35" s="2" t="inlineStr">
         <is>
           <t>eero Mesh Router (3-Pack)</t>
         </is>
@@ -1929,12 +2032,12 @@
           <t>https://www.bestbuy.com/site/eero-6-ax1800-dual-band-mesh-wi-fi-6-system-3-pack-white/6433419.p?skuId=6433419</t>
         </is>
       </c>
-      <c r="G35" s="1" t="inlineStr">
+      <c r="G35" s="2" t="inlineStr">
         <is>
           <t>6433419</t>
         </is>
       </c>
-      <c r="H35" s="1" t="inlineStr">
+      <c r="H35" s="2" t="inlineStr">
         <is>
           <t>Currently Active</t>
         </is>
@@ -1942,11 +2045,14 @@
       <c r="I35" s="7" t="n">
         <v>139.99</v>
       </c>
-      <c r="J35" s="1" t="n">
+      <c r="J35" s="2" t="n">
         <v>139.99</v>
       </c>
-      <c r="K35" s="1" t="n"/>
+      <c r="K35" s="2" t="n"/>
       <c r="L35" s="13" t="n">
+        <v>139.99</v>
+      </c>
+      <c r="M35" s="13" t="n">
         <v>139.99</v>
       </c>
     </row>
@@ -1957,15 +2063,15 @@
       <c r="B36" s="10" t="n">
         <v>0</v>
       </c>
-      <c r="C36" s="1" t="n">
+      <c r="C36" s="2" t="n">
         <v>467</v>
       </c>
-      <c r="D36" s="1" t="inlineStr">
+      <c r="D36" s="2" t="inlineStr">
         <is>
           <t>Router</t>
         </is>
       </c>
-      <c r="E36" s="1" t="inlineStr">
+      <c r="E36" s="2" t="inlineStr">
         <is>
           <t>eero Mesh Wi-Fi Router</t>
         </is>
@@ -1975,12 +2081,12 @@
           <t>https://www.bestbuy.com/product/eero-6-dual-band-mesh-wi-fi-6-router-1-pack-white/J39QV832QV/sku/6433416#tabbed-customerreviews</t>
         </is>
       </c>
-      <c r="G36" s="1" t="inlineStr">
+      <c r="G36" s="2" t="inlineStr">
         <is>
           <t>6433416</t>
         </is>
       </c>
-      <c r="H36" s="1" t="inlineStr">
+      <c r="H36" s="2" t="inlineStr">
         <is>
           <t>Currently Active</t>
         </is>
@@ -1995,6 +2101,9 @@
       <c r="L36" s="13" t="n">
         <v>89.98999999999999</v>
       </c>
+      <c r="M36" s="13" t="n">
+        <v>89.98999999999999</v>
+      </c>
     </row>
     <row r="37" ht="15.75" customHeight="1" s="11">
       <c r="A37" s="9" t="n">
@@ -2003,15 +2112,15 @@
       <c r="B37" s="10" t="n">
         <v>0</v>
       </c>
-      <c r="C37" s="1" t="n">
+      <c r="C37" s="2" t="n">
         <v>526</v>
       </c>
-      <c r="D37" s="1" t="inlineStr">
+      <c r="D37" s="2" t="inlineStr">
         <is>
           <t>Subwoofer</t>
         </is>
       </c>
-      <c r="E37" s="1" t="inlineStr">
+      <c r="E37" s="2" t="inlineStr">
         <is>
           <t>Sony 300w Wireless Subwoofer</t>
         </is>
@@ -2021,12 +2130,12 @@
           <t>https://www.bestbuy.com/site/sony-sa-sw3-200w-wireless-subwoofer-black/6467459.p?skuId=6467459</t>
         </is>
       </c>
-      <c r="G37" s="1" t="inlineStr">
+      <c r="G37" s="2" t="inlineStr">
         <is>
           <t>6467459</t>
         </is>
       </c>
-      <c r="H37" s="1" t="inlineStr">
+      <c r="H37" s="2" t="inlineStr">
         <is>
           <t>Currently Active</t>
         </is>
@@ -2041,6 +2150,9 @@
       <c r="L37" s="13" t="n">
         <v>349.99</v>
       </c>
+      <c r="M37" s="13" t="n">
+        <v>349.99</v>
+      </c>
     </row>
     <row r="38" ht="15.75" customHeight="1" s="11">
       <c r="A38" s="9" t="n">
@@ -2049,15 +2161,15 @@
       <c r="B38" s="10" t="n">
         <v>0</v>
       </c>
-      <c r="C38" s="1" t="n">
+      <c r="C38" s="2" t="n">
         <v>527</v>
       </c>
-      <c r="D38" s="1" t="inlineStr">
+      <c r="D38" s="2" t="inlineStr">
         <is>
           <t>Subwoofer</t>
         </is>
       </c>
-      <c r="E38" s="1" t="inlineStr">
+      <c r="E38" s="2" t="inlineStr">
         <is>
           <t>Bose Bass Module Home Theater Subwoofer</t>
         </is>
@@ -2067,12 +2179,12 @@
           <t>https://www.bestbuy.com/site/bose-bass-module-700-wireless-home-theater-subwoofer-black/6280563.p?skuId=6280563</t>
         </is>
       </c>
-      <c r="G38" s="1" t="inlineStr">
+      <c r="G38" s="2" t="inlineStr">
         <is>
           <t>6280563</t>
         </is>
       </c>
-      <c r="H38" s="1" t="inlineStr">
+      <c r="H38" s="2" t="inlineStr">
         <is>
           <t>Currently Active</t>
         </is>
@@ -2087,6 +2199,9 @@
       <c r="L38" s="13" t="n">
         <v>899.99</v>
       </c>
+      <c r="M38" s="13" t="n">
+        <v>899.99</v>
+      </c>
     </row>
     <row r="39" ht="15.75" customHeight="1" s="11">
       <c r="A39" s="9" t="n">
@@ -2095,15 +2210,15 @@
       <c r="B39" s="10" t="n">
         <v>-0.04</v>
       </c>
-      <c r="C39" s="1" t="n">
+      <c r="C39" s="2" t="n">
         <v>554</v>
       </c>
-      <c r="D39" s="1" t="inlineStr">
+      <c r="D39" s="2" t="inlineStr">
         <is>
           <t>Toaster</t>
         </is>
       </c>
-      <c r="E39" s="1" t="inlineStr">
+      <c r="E39" s="2" t="inlineStr">
         <is>
           <t>Breville Convection Toaster Oven with Air Fryer</t>
         </is>
@@ -2113,12 +2228,12 @@
           <t>https://www.bestbuy.com/product/breville-smart-oven-air-fryer-compact-0-5-cubic-feet-toaster-oven-brushed-stainless-steel/J7266LFC5K/sku/6617568</t>
         </is>
       </c>
-      <c r="G39" s="1" t="inlineStr">
+      <c r="G39" s="2" t="inlineStr">
         <is>
           <t>6617568</t>
         </is>
       </c>
-      <c r="H39" s="1" t="inlineStr">
+      <c r="H39" s="2" t="inlineStr">
         <is>
           <t>Currently Active</t>
         </is>
@@ -2133,6 +2248,9 @@
       <c r="L39" s="13" t="n">
         <v>199.95</v>
       </c>
+      <c r="M39" s="13" t="n">
+        <v>199.95</v>
+      </c>
     </row>
     <row r="40" ht="15.75" customHeight="1" s="11">
       <c r="A40" s="9" t="n">
@@ -2141,15 +2259,15 @@
       <c r="B40" s="10" t="n">
         <v>-50</v>
       </c>
-      <c r="C40" s="1" t="n">
+      <c r="C40" s="2" t="n">
         <v>565</v>
       </c>
-      <c r="D40" s="1" t="inlineStr">
+      <c r="D40" s="2" t="inlineStr">
         <is>
           <t>TV</t>
         </is>
       </c>
-      <c r="E40" s="1" t="inlineStr">
+      <c r="E40" s="2" t="inlineStr">
         <is>
           <t>Samsung 65" OLED UHD Smart TV</t>
         </is>
@@ -2159,12 +2277,12 @@
           <t>https://www.bestbuy.com/product/samsung-65-class-s84f-oled-4k-uhd-vision-ai-smart-tizen-tv-2025/JJGRF39ZVL/sku/6643538</t>
         </is>
       </c>
-      <c r="G40" s="1" t="inlineStr">
+      <c r="G40" s="2" t="inlineStr">
         <is>
           <t>6643538</t>
         </is>
       </c>
-      <c r="H40" s="1" t="inlineStr">
+      <c r="H40" s="2" t="inlineStr">
         <is>
           <t>Currently Active</t>
         </is>
@@ -2179,17 +2297,20 @@
       <c r="L40" s="15" t="n">
         <v>849.99</v>
       </c>
+      <c r="M40" s="15" t="n">
+        <v>849.99</v>
+      </c>
     </row>
     <row r="41" ht="15.75" customHeight="1" s="11">
-      <c r="C41" s="1" t="n">
+      <c r="C41" s="2" t="n">
         <v>566</v>
       </c>
-      <c r="D41" s="1" t="inlineStr">
+      <c r="D41" s="2" t="inlineStr">
         <is>
           <t>TV</t>
         </is>
       </c>
-      <c r="E41" s="1" t="inlineStr">
+      <c r="E41" s="2" t="inlineStr">
         <is>
           <t>LG 65" 4K LED TV</t>
         </is>
@@ -2202,7 +2323,7 @@
       <c r="G41" s="8" t="n">
         <v>6593578</v>
       </c>
-      <c r="H41" s="1" t="inlineStr">
+      <c r="H41" s="2" t="inlineStr">
         <is>
           <t>Currently Active</t>
         </is>
@@ -2214,6 +2335,9 @@
       <c r="L41" s="13" t="n">
         <v>599.99</v>
       </c>
+      <c r="M41" s="13" t="n">
+        <v>599.99</v>
+      </c>
     </row>
     <row r="42" ht="15.75" customHeight="1" s="11">
       <c r="A42" s="9" t="n">
@@ -2222,15 +2346,15 @@
       <c r="B42" s="10" t="n">
         <v>0</v>
       </c>
-      <c r="C42" s="1" t="n">
+      <c r="C42" s="2" t="n">
         <v>567</v>
       </c>
-      <c r="D42" s="1" t="inlineStr">
+      <c r="D42" s="2" t="inlineStr">
         <is>
           <t>TV</t>
         </is>
       </c>
-      <c r="E42" s="1" t="inlineStr">
+      <c r="E42" s="2" t="inlineStr">
         <is>
           <t>LG 55" OLED Smart TV</t>
         </is>
@@ -2240,12 +2364,12 @@
           <t>https://www.bestbuy.com/product/lg-55-class-b5-series-oled-ai-4k-uhd-smart-webos-tv-2025/JJ8VPZTKH9/sku/6635751?utm_source=feed?extStoreId=1767&amp;ref=212&amp;loc=19551139597&amp;gclsrc=aw.ds&amp;gad_source=1&amp;gad_campaignid=19550235539&amp;gbraid=0AAAAAD-ORIhGp7TyBq_YUtG8pO</t>
         </is>
       </c>
-      <c r="G42" s="1" t="inlineStr">
+      <c r="G42" s="2" t="inlineStr">
         <is>
           <t>6635751</t>
         </is>
       </c>
-      <c r="H42" s="1" t="inlineStr">
+      <c r="H42" s="2" t="inlineStr">
         <is>
           <t>Currently Active</t>
         </is>
@@ -2260,17 +2384,20 @@
       <c r="L42" s="13" t="n">
         <v>899.99</v>
       </c>
+      <c r="M42" s="13" t="n">
+        <v>899.99</v>
+      </c>
     </row>
     <row r="43" ht="15.75" customHeight="1" s="11">
-      <c r="C43" s="1" t="n">
+      <c r="C43" s="2" t="n">
         <v>569</v>
       </c>
-      <c r="D43" s="1" t="inlineStr">
+      <c r="D43" s="2" t="inlineStr">
         <is>
           <t>TV</t>
         </is>
       </c>
-      <c r="E43" s="1" t="inlineStr">
+      <c r="E43" s="2" t="inlineStr">
         <is>
           <t>Samsung 43" QLED TV</t>
         </is>
@@ -2283,7 +2410,7 @@
       <c r="G43" s="8" t="n">
         <v>6617420</v>
       </c>
-      <c r="H43" s="1" t="inlineStr">
+      <c r="H43" s="2" t="inlineStr">
         <is>
           <t>Currently Active</t>
         </is>
@@ -2295,6 +2422,9 @@
       <c r="L43" s="15" t="n">
         <v>399.99</v>
       </c>
+      <c r="M43" s="15" t="n">
+        <v>399.99</v>
+      </c>
     </row>
     <row r="44" ht="15.75" customHeight="1" s="11">
       <c r="A44" s="4" t="n">
@@ -2303,15 +2433,15 @@
       <c r="B44" s="5" t="n">
         <v>0</v>
       </c>
-      <c r="C44" s="1" t="n">
+      <c r="C44" s="2" t="n">
         <v>570</v>
       </c>
-      <c r="D44" s="1" t="inlineStr">
+      <c r="D44" s="2" t="inlineStr">
         <is>
           <t>TV</t>
         </is>
       </c>
-      <c r="E44" s="1" t="inlineStr">
+      <c r="E44" s="2" t="inlineStr">
         <is>
           <t>Sony 43" Smart LED TV</t>
         </is>
@@ -2321,12 +2451,12 @@
           <t>https://www.bestbuy.com/site/sony-43-class-bravia-3-led-4k-uhd-smart-google-tv-2024/6578580.p?skuId=6578580</t>
         </is>
       </c>
-      <c r="G44" s="1" t="inlineStr">
+      <c r="G44" s="2" t="inlineStr">
         <is>
           <t>6578580</t>
         </is>
       </c>
-      <c r="H44" s="1" t="inlineStr">
+      <c r="H44" s="2" t="inlineStr">
         <is>
           <t>Currently Active</t>
         </is>
@@ -2334,13 +2464,16 @@
       <c r="I44" s="7" t="n">
         <v>499.99</v>
       </c>
-      <c r="J44" s="1" t="n">
+      <c r="J44" s="2" t="n">
         <v>499.99</v>
       </c>
       <c r="K44" s="4" t="n">
         <v>499.99</v>
       </c>
       <c r="L44" s="13" t="n">
+        <v>499.99</v>
+      </c>
+      <c r="M44" s="13" t="n">
         <v>499.99</v>
       </c>
     </row>
@@ -2351,15 +2484,15 @@
       <c r="B45" s="10" t="n">
         <v>0</v>
       </c>
-      <c r="C45" s="1" t="n">
+      <c r="C45" s="2" t="n">
         <v>572</v>
       </c>
-      <c r="D45" s="1" t="inlineStr">
+      <c r="D45" s="2" t="inlineStr">
         <is>
           <t>TV</t>
         </is>
       </c>
-      <c r="E45" s="1" t="inlineStr">
+      <c r="E45" s="2" t="inlineStr">
         <is>
           <t>Samsung 50" 4K LED TV</t>
         </is>
@@ -2369,12 +2502,12 @@
           <t>https://www.bestbuy.com/product/samsung-50-class-q7f-series-qled-4k-uhd-samsungvision-ai-smart-tizen-tv-2025/J3ZYGXCP6Q/sku/6619441?utm_source=feed?extStoreId=894&amp;ref=212&amp;loc=TVsGeneral&amp;gclsrc=aw.ds&amp;gad_source=1&amp;gad_campaignid=20758864463&amp;gbraid=0AAAAAD-O</t>
         </is>
       </c>
-      <c r="G45" s="1" t="inlineStr">
+      <c r="G45" s="2" t="inlineStr">
         <is>
           <t>6619441</t>
         </is>
       </c>
-      <c r="H45" s="1" t="inlineStr">
+      <c r="H45" s="2" t="inlineStr">
         <is>
           <t>Currently Active</t>
         </is>
@@ -2389,6 +2522,9 @@
       <c r="L45" s="13" t="n">
         <v>379.99</v>
       </c>
+      <c r="M45" s="13" t="n">
+        <v>379.99</v>
+      </c>
     </row>
     <row r="46" ht="15.75" customHeight="1" s="11">
       <c r="A46" s="4" t="n">
@@ -2397,15 +2533,15 @@
       <c r="B46" s="5" t="n">
         <v>0</v>
       </c>
-      <c r="C46" s="1" t="n">
+      <c r="C46" s="2" t="n">
         <v>574</v>
       </c>
-      <c r="D46" s="1" t="inlineStr">
+      <c r="D46" s="2" t="inlineStr">
         <is>
           <t>TV</t>
         </is>
       </c>
-      <c r="E46" s="1" t="inlineStr">
+      <c r="E46" s="2" t="inlineStr">
         <is>
           <t>Sony 65" Smart 4K LED TV</t>
         </is>
@@ -2415,12 +2551,12 @@
           <t>https://www.bestbuy.com/site/sony-65-class-bravia-3-led-4k-uhd-smart-google-tv-2024/6578579.p?skuId=6578579</t>
         </is>
       </c>
-      <c r="G46" s="1" t="inlineStr">
+      <c r="G46" s="2" t="inlineStr">
         <is>
           <t>6578579</t>
         </is>
       </c>
-      <c r="H46" s="1" t="inlineStr">
+      <c r="H46" s="2" t="inlineStr">
         <is>
           <t>Currently Active</t>
         </is>
@@ -2428,13 +2564,16 @@
       <c r="I46" s="7" t="n">
         <v>649.99</v>
       </c>
-      <c r="J46" s="1" t="n">
+      <c r="J46" s="2" t="n">
         <v>649.99</v>
       </c>
       <c r="K46" s="4" t="n">
         <v>649.99</v>
       </c>
       <c r="L46" s="13" t="n">
+        <v>649.99</v>
+      </c>
+      <c r="M46" s="13" t="n">
         <v>649.99</v>
       </c>
     </row>
@@ -2445,15 +2584,15 @@
       <c r="B47" s="10" t="n">
         <v>0</v>
       </c>
-      <c r="C47" s="1" t="n">
+      <c r="C47" s="2" t="n">
         <v>577</v>
       </c>
-      <c r="D47" s="1" t="inlineStr">
+      <c r="D47" s="2" t="inlineStr">
         <is>
           <t>TV</t>
         </is>
       </c>
-      <c r="E47" s="1" t="inlineStr">
+      <c r="E47" s="2" t="inlineStr">
         <is>
           <t>TCL 32" 1080p LED TV</t>
         </is>
@@ -2463,12 +2602,12 @@
           <t>https://www.bestbuy.com/product/tcl-32-class-q3k-series-1080p-fhd-qled-smart-tv-with-google-tv-2025/J36QYTQZCY/sku/6625838</t>
         </is>
       </c>
-      <c r="G47" s="1" t="inlineStr">
+      <c r="G47" s="2" t="inlineStr">
         <is>
           <t>6625838</t>
         </is>
       </c>
-      <c r="H47" s="1" t="inlineStr">
+      <c r="H47" s="2" t="inlineStr">
         <is>
           <t>Currently Active</t>
         </is>
@@ -2483,17 +2622,20 @@
       <c r="L47" s="13" t="n">
         <v>139.99</v>
       </c>
+      <c r="M47" s="13" t="n">
+        <v>139.99</v>
+      </c>
     </row>
     <row r="48" ht="15.75" customHeight="1" s="11">
-      <c r="C48" s="1" t="n">
+      <c r="C48" s="2" t="n">
         <v>578</v>
       </c>
-      <c r="D48" s="1" t="inlineStr">
+      <c r="D48" s="2" t="inlineStr">
         <is>
           <t>TV</t>
         </is>
       </c>
-      <c r="E48" s="1" t="inlineStr">
+      <c r="E48" s="2" t="inlineStr">
         <is>
           <t>Samsung 32" 1080p LED TV</t>
         </is>
@@ -2506,7 +2648,7 @@
       <c r="G48" s="8" t="n">
         <v>6617418</v>
       </c>
-      <c r="H48" s="1" t="inlineStr">
+      <c r="H48" s="2" t="inlineStr">
         <is>
           <t>Currently Active</t>
         </is>
@@ -2518,6 +2660,9 @@
       <c r="L48" s="13" t="n">
         <v>399.99</v>
       </c>
+      <c r="M48" s="13" t="n">
+        <v>399.99</v>
+      </c>
     </row>
     <row r="49" ht="15.75" customHeight="1" s="11">
       <c r="A49" s="9" t="n">
@@ -2526,15 +2671,15 @@
       <c r="B49" s="10" t="n">
         <v>0</v>
       </c>
-      <c r="C49" s="1" t="n">
+      <c r="C49" s="2" t="n">
         <v>586</v>
       </c>
-      <c r="D49" s="1" t="inlineStr">
+      <c r="D49" s="2" t="inlineStr">
         <is>
           <t>TV</t>
         </is>
       </c>
-      <c r="E49" s="1" t="inlineStr">
+      <c r="E49" s="2" t="inlineStr">
         <is>
           <t>TCL 32" 1080p LED TV</t>
         </is>
@@ -2544,12 +2689,12 @@
           <t>https://www.bestbuy.com/product/tcl-32-class-q3k-series-1080p-fhd-qled-smart-tv-with-google-tv-2025/J36QYTQZCY/sku/6625838</t>
         </is>
       </c>
-      <c r="G49" s="1" t="inlineStr">
+      <c r="G49" s="2" t="inlineStr">
         <is>
           <t>6625838</t>
         </is>
       </c>
-      <c r="H49" s="1" t="inlineStr">
+      <c r="H49" s="2" t="inlineStr">
         <is>
           <t>Currently Active</t>
         </is>
@@ -2564,6 +2709,9 @@
       <c r="L49" s="13" t="n">
         <v>139.99</v>
       </c>
+      <c r="M49" s="13" t="n">
+        <v>139.99</v>
+      </c>
     </row>
     <row r="50" ht="15.75" customHeight="1" s="11">
       <c r="A50" s="9" t="n">
@@ -2572,15 +2720,15 @@
       <c r="B50" s="10" t="n">
         <v>0</v>
       </c>
-      <c r="C50" s="1" t="n">
+      <c r="C50" s="2" t="n">
         <v>587</v>
       </c>
-      <c r="D50" s="1" t="inlineStr">
+      <c r="D50" s="2" t="inlineStr">
         <is>
           <t>TV</t>
         </is>
       </c>
-      <c r="E50" s="1" t="inlineStr">
+      <c r="E50" s="2" t="inlineStr">
         <is>
           <t>LG 48" OLED UHD Smart TV</t>
         </is>
@@ -2590,12 +2738,12 @@
           <t>https://www.bestbuy.com/product/lg-48-class-b5-series-oled-ai-4k-uhd-smart-webos-tv-2025/JJ8VPZTK9F/sku/6635292</t>
         </is>
       </c>
-      <c r="G50" s="1" t="inlineStr">
+      <c r="G50" s="2" t="inlineStr">
         <is>
           <t>6635292</t>
         </is>
       </c>
-      <c r="H50" s="1" t="inlineStr">
+      <c r="H50" s="2" t="inlineStr">
         <is>
           <t>Currently Active</t>
         </is>
@@ -2610,17 +2758,20 @@
       <c r="L50" s="13" t="n">
         <v>599.99</v>
       </c>
+      <c r="M50" s="13" t="n">
+        <v>599.99</v>
+      </c>
     </row>
     <row r="51" ht="15.75" customHeight="1" s="11">
-      <c r="C51" s="1" t="n">
+      <c r="C51" s="2" t="n">
         <v>590</v>
       </c>
-      <c r="D51" s="1" t="inlineStr">
+      <c r="D51" s="2" t="inlineStr">
         <is>
           <t>TV</t>
         </is>
       </c>
-      <c r="E51" s="1" t="inlineStr">
+      <c r="E51" s="2" t="inlineStr">
         <is>
           <t>Samsung 75" 4K LED TV</t>
         </is>
@@ -2633,7 +2784,7 @@
       <c r="G51" s="8" t="n">
         <v>6619142</v>
       </c>
-      <c r="H51" s="1" t="inlineStr">
+      <c r="H51" s="2" t="inlineStr">
         <is>
           <t>Currently Active</t>
         </is>
@@ -2645,17 +2796,20 @@
       <c r="L51" s="13" t="n">
         <v>699.99</v>
       </c>
+      <c r="M51" s="13" t="n">
+        <v>699.99</v>
+      </c>
     </row>
     <row r="52" ht="15.75" customHeight="1" s="11">
-      <c r="C52" s="1" t="n">
+      <c r="C52" s="2" t="n">
         <v>592</v>
       </c>
-      <c r="D52" s="1" t="inlineStr">
+      <c r="D52" s="2" t="inlineStr">
         <is>
           <t>TV</t>
         </is>
       </c>
-      <c r="E52" s="1" t="inlineStr">
+      <c r="E52" s="2" t="inlineStr">
         <is>
           <t>LG 75" 4K QNED TV</t>
         </is>
@@ -2668,7 +2822,7 @@
       <c r="G52" s="8" t="n">
         <v>6621816</v>
       </c>
-      <c r="H52" s="1" t="inlineStr">
+      <c r="H52" s="2" t="inlineStr">
         <is>
           <t>Currently Active</t>
         </is>
@@ -2680,6 +2834,9 @@
       <c r="L52" s="15" t="n">
         <v>899.99</v>
       </c>
+      <c r="M52" s="15" t="n">
+        <v>899.99</v>
+      </c>
     </row>
     <row r="53" ht="15.75" customHeight="1" s="11">
       <c r="A53" s="9" t="n">
@@ -2688,15 +2845,15 @@
       <c r="B53" s="10" t="n">
         <v>0.99</v>
       </c>
-      <c r="C53" s="1" t="n">
+      <c r="C53" s="2" t="n">
         <v>595</v>
       </c>
-      <c r="D53" s="1" t="inlineStr">
+      <c r="D53" s="2" t="inlineStr">
         <is>
           <t>TV</t>
         </is>
       </c>
-      <c r="E53" s="1" t="inlineStr">
+      <c r="E53" s="2" t="inlineStr">
         <is>
           <t>LG 24" LED TV</t>
         </is>
@@ -2706,12 +2863,12 @@
           <t>https://www.bestbuy.com/site/lg-24-class-led-hd-smart-tv-with-webos-2022/6506779.p?skuId=6506779</t>
         </is>
       </c>
-      <c r="G53" s="1" t="inlineStr">
+      <c r="G53" s="2" t="inlineStr">
         <is>
           <t>6506779</t>
         </is>
       </c>
-      <c r="H53" s="1" t="inlineStr">
+      <c r="H53" s="2" t="inlineStr">
         <is>
           <t>Currently Active</t>
         </is>
@@ -2726,6 +2883,9 @@
       <c r="L53" s="13" t="n">
         <v>169.99</v>
       </c>
+      <c r="M53" s="13" t="n">
+        <v>169.99</v>
+      </c>
     </row>
     <row r="54" ht="15.75" customHeight="1" s="11">
       <c r="A54" s="9" t="n">
@@ -2734,15 +2894,15 @@
       <c r="B54" s="10" t="n">
         <v>0</v>
       </c>
-      <c r="C54" s="1" t="n">
+      <c r="C54" s="2" t="n">
         <v>647</v>
       </c>
-      <c r="D54" s="1" t="inlineStr">
+      <c r="D54" s="2" t="inlineStr">
         <is>
           <t>Window Air Conditioner</t>
         </is>
       </c>
-      <c r="E54" s="1" t="inlineStr">
+      <c r="E54" s="2" t="inlineStr">
         <is>
           <t>LG 23,000 BTU Window Air Conditioner</t>
         </is>
@@ -2752,12 +2912,12 @@
           <t>https://www.bestbuy.com/product/lg-1400-sq-ft-23000-btu-230v-smart-window-air-conditioner-with-heat-white/J7G5655ZYX/sku/6589451?utm_source=feed?extStoreId=&amp;ref=212&amp;loc=20482168767&amp;gclsrc=aw.ds&amp;gad_source=1&amp;gad_campaignid=20482183434&amp;gbraid=0AAAAAD-ORIiC5</t>
         </is>
       </c>
-      <c r="G54" s="1" t="inlineStr">
+      <c r="G54" s="2" t="inlineStr">
         <is>
           <t>6589451</t>
         </is>
       </c>
-      <c r="H54" s="1" t="inlineStr">
+      <c r="H54" s="2" t="inlineStr">
         <is>
           <t>Currently Active</t>
         </is>
@@ -2770,6 +2930,9 @@
         <v>799.99</v>
       </c>
       <c r="L54" s="13" t="n">
+        <v>799.99</v>
+      </c>
+      <c r="M54" s="13" t="n">
         <v>799.99</v>
       </c>
     </row>

</xml_diff>